<commit_message>
S1 to S3 98% done
</commit_message>
<xml_diff>
--- a/life-inforce-tool/reference_files/product_characteristics.xlsx
+++ b/life-inforce-tool/reference_files/product_characteristics.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafi_\OneDrive\Bureau\NETAC\desjardins-tools\life-inforce-tool\reference_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C8EF65B-CB53-48E9-B74E-58FAA7ABBB0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5207687-6239-448E-A23A-628E412A921D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="1620" windowWidth="29040" windowHeight="15720" xr2:uid="{8C2A5375-7FA4-4E2C-80BA-7804EEAE4A5C}"/>
   </bookViews>
   <sheets>
     <sheet name="characteristics" sheetId="1" r:id="rId1"/>
     <sheet name="legend" sheetId="2" r:id="rId2"/>
+    <sheet name="to_json" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="59">
   <si>
     <t>id</t>
   </si>
@@ -208,6 +209,15 @@
   </si>
   <si>
     <t>premium never ends</t>
+  </si>
+  <si>
+    <t>joint_type</t>
+  </si>
+  <si>
+    <t>Joint</t>
+  </si>
+  <si>
+    <t>joint_age_equivalent</t>
   </si>
 </sst>
 </file>
@@ -612,7 +622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99BF2FC8-1AD7-404A-A635-34F6D4CEECC1}">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
@@ -621,14 +631,16 @@
     <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="31.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="31.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="58.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="8" max="8" width="22.5703125" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="31.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="58.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -648,22 +660,28 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -682,23 +700,25 @@
       <c r="F2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" s="2">
-        <v>85</v>
-      </c>
-      <c r="I2" s="2">
-        <v>85</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K2" s="2" t="s">
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="2">
+        <v>85</v>
+      </c>
+      <c r="K2" s="2">
+        <v>85</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>19</v>
       </c>
@@ -717,23 +737,25 @@
       <c r="F3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" s="2">
-        <v>85</v>
-      </c>
-      <c r="I3" s="2">
-        <v>85</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K3" s="2" t="s">
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="2">
+        <v>85</v>
+      </c>
+      <c r="K3" s="2">
+        <v>85</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M3" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>22</v>
       </c>
@@ -752,23 +774,25 @@
       <c r="F4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" s="2">
-        <v>85</v>
-      </c>
-      <c r="I4" s="2">
-        <v>85</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K4" s="2" t="s">
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="2">
+        <v>85</v>
+      </c>
+      <c r="K4" s="2">
+        <v>85</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M4" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>25</v>
       </c>
@@ -787,23 +811,25 @@
       <c r="F5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H5" s="2">
-        <v>85</v>
-      </c>
-      <c r="I5" s="2">
-        <v>85</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K5" s="2" t="s">
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" s="2">
+        <v>85</v>
+      </c>
+      <c r="K5" s="2">
+        <v>85</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M5" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
@@ -822,23 +848,25 @@
       <c r="F6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H6" s="2">
-        <v>85</v>
-      </c>
-      <c r="I6" s="2">
-        <v>85</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K6" s="2" t="s">
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" s="2">
+        <v>85</v>
+      </c>
+      <c r="K6" s="2">
+        <v>85</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
@@ -857,23 +885,25 @@
       <c r="F7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" s="2">
-        <v>85</v>
-      </c>
-      <c r="I7" s="2">
-        <v>85</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K7" s="2" t="s">
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J7" s="2">
+        <v>85</v>
+      </c>
+      <c r="K7" s="2">
+        <v>85</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M7" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>34</v>
       </c>
@@ -890,25 +920,31 @@
         <v>15</v>
       </c>
       <c r="F8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" s="2">
-        <v>85</v>
-      </c>
-      <c r="I8" s="2">
-        <v>85</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K8" s="2" t="s">
+      <c r="H8" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J8" s="2">
+        <v>85</v>
+      </c>
+      <c r="K8" s="2">
+        <v>85</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M8" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>37</v>
       </c>
@@ -925,25 +961,31 @@
         <v>15</v>
       </c>
       <c r="F9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" s="2">
-        <v>85</v>
-      </c>
-      <c r="I9" s="2">
-        <v>85</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K9" s="2" t="s">
+      <c r="H9" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J9" s="2">
+        <v>85</v>
+      </c>
+      <c r="K9" s="2">
+        <v>85</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M9" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>39</v>
       </c>
@@ -960,25 +1002,31 @@
         <v>15</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H10" s="2">
-        <v>85</v>
-      </c>
-      <c r="I10" s="2">
-        <v>85</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K10" s="2" t="s">
+      <c r="H10" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J10" s="2">
+        <v>85</v>
+      </c>
+      <c r="K10" s="2">
+        <v>85</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M10" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>41</v>
       </c>
@@ -995,25 +1043,31 @@
         <v>15</v>
       </c>
       <c r="F11" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H11" s="2">
-        <v>85</v>
-      </c>
-      <c r="I11" s="2">
-        <v>85</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K11" s="2" t="s">
+      <c r="H11" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J11" s="2">
+        <v>85</v>
+      </c>
+      <c r="K11" s="2">
+        <v>85</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M11" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>43</v>
       </c>
@@ -1030,25 +1084,31 @@
         <v>15</v>
       </c>
       <c r="F12" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H12" s="2">
-        <v>85</v>
-      </c>
-      <c r="I12" s="2">
-        <v>85</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K12" s="2" t="s">
+      <c r="H12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J12" s="2">
+        <v>85</v>
+      </c>
+      <c r="K12" s="2">
+        <v>85</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M12" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>45</v>
       </c>
@@ -1065,21 +1125,27 @@
         <v>15</v>
       </c>
       <c r="F13" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H13" s="2">
-        <v>85</v>
-      </c>
-      <c r="I13" s="2">
-        <v>85</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K13" s="2" t="s">
+      <c r="H13" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J13" s="2">
+        <v>85</v>
+      </c>
+      <c r="K13" s="2">
+        <v>85</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M13" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1178,4 +1244,98 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6703E102-F93D-4445-A900-5FF358402C9E}">
+  <dimension ref="A1:A14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="str">
+        <f>_xlfn.TEXTJOIN(" | ", FALSE,characteristics!A1:M1)</f>
+        <v>id | product_type | plan_name | coverage_plan_code | rate_scale | coverage_type | joint_type | joint_age_equivalent | expiration_type | end_of_premium_age_or_duration | end_of_coverage_age_or_duration | end_of_premium_type | base_premium_rate_band</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="str">
+        <f>_xlfn.TEXTJOIN(" | ", FALSE,characteristics!A2:M2)</f>
+        <v>LT10IB | Term | Life Term 10 | LT10I | B | Individual |  |  | C | 85 | 85 | C | B00025; B00050; B00100; B00250; B00500; B01000; B02000; B10000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="str">
+        <f>_xlfn.TEXTJOIN(" | ", FALSE,characteristics!A3:M3)</f>
+        <v>LT15IB | Term | Life Term 15 | LT15I | B | Individual |  |  | C | 85 | 85 | C | B00025; B00050; B00100; B00250; B00500; B01000; B02000; B10000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="str">
+        <f>_xlfn.TEXTJOIN(" | ", FALSE,characteristics!A4:M4)</f>
+        <v>LT20IB | Term | Life Term 20 | LT20I | B | Individual |  |  | C | 85 | 85 | C | B00025; B00050; B00100; B00250; B00500; B01000; B02000; B10000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="str">
+        <f>_xlfn.TEXTJOIN(" | ", FALSE,characteristics!A5:M5)</f>
+        <v>LT25IB | Term | Life Term 25 | LT25I | B | Individual |  |  | C | 85 | 85 | C | B00025; B00050; B00100; B00250; B00500; B01000; B02000; B10000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="str">
+        <f>_xlfn.TEXTJOIN(" | ", FALSE,characteristics!A6:M6)</f>
+        <v>LT30IB | Term | Life Term 30 | LT30I | B | Individual |  |  | C | 85 | 85 | C | B00025; B00050; B00100; B00250; B00500; B01000; B02000; B10000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="str">
+        <f>_xlfn.TEXTJOIN(" | ", FALSE,characteristics!A7:M7)</f>
+        <v>LT65IB | Term | Life Term to 65 | LT65I | B | Individual |  |  | C | 85 | 85 | C | B00025; B00050; B00100; B00250; B00500; B01000; B02000; B10000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="str">
+        <f>_xlfn.TEXTJOIN(" | ", FALSE,characteristics!A8:M8)</f>
+        <v>LT10FB | Term | Life Term 10 | LT10F | B | Joint | JFTD | FALSE | C | 85 | 85 | C | B00025; B00050; B00100; B00250; B00500; B01000; B02000; B10000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="str">
+        <f>_xlfn.TEXTJOIN(" | ", FALSE,characteristics!A9:M9)</f>
+        <v>LT15FB | Term | Life Term 15 | LT15F | B | Joint | JFTD | FALSE | C | 85 | 85 | C | B00025; B00050; B00100; B00250; B00500; B01000; B02000; B10000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="str">
+        <f>_xlfn.TEXTJOIN(" | ", FALSE,characteristics!A10:M10)</f>
+        <v>LT20FB | Term | Life Term 20 | LT20F | B | Joint | JFTD | FALSE | C | 85 | 85 | C | B00025; B00050; B00100; B00250; B00500; B01000; B02000; B10000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="str">
+        <f>_xlfn.TEXTJOIN(" | ", FALSE,characteristics!A11:M11)</f>
+        <v>LT25FB | Term | Life Term 25 | LT25F | B | Joint | JFTD | FALSE | C | 85 | 85 | C | B00025; B00050; B00100; B00250; B00500; B01000; B02000; B10000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="str">
+        <f>_xlfn.TEXTJOIN(" | ", FALSE,characteristics!A12:M12)</f>
+        <v>LT30FB | Term | Life Term 30 | LT30F | B | Joint | JFTD | FALSE | C | 85 | 85 | C | B00025; B00050; B00100; B00250; B00500; B01000; B02000; B10000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="str">
+        <f>_xlfn.TEXTJOIN(" | ", FALSE,characteristics!A13:M13)</f>
+        <v>LT65FB | Term | Life Term to 65 | LT65F | B | Joint | JFTD | FALSE | C | 85 | 85 | C | B00025; B00050; B00100; B00250; B00500; B01000; B02000; B10000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="str">
+        <f>_xlfn.TEXTJOIN(" | ", FALSE,characteristics!A14:M14)</f>
+        <v xml:space="preserve"> |  |  |  |  |  |  |  |  |  |  |  | </v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>